<commit_message>
added all apps menu, updated buttons on top right of all apps and updated excel
</commit_message>
<xml_diff>
--- a/public/excel/BTS SIO 2025 - E4 - Tableau de synthèse - Joao.xlsx
+++ b/public/excel/BTS SIO 2025 - E4 - Tableau de synthèse - Joao.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jalmeidasantos\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\webshell-portfolio\public\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACF203F1-97E2-446B-8D9C-6661D7A12D0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EBC1005-5A59-4FB0-8FFB-86569FB74AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -194,6 +194,9 @@
   </si>
   <si>
     <t>Création d'une application fullstack (C# .NET &amp; Angular) pour gérer le stock d'un Fastfood (Apprentisage)</t>
+  </si>
+  <si>
+    <t>Création d'une application de gestion de température/lumière/ventilation etc des bureaux d'un batiment</t>
   </si>
 </sst>
 </file>
@@ -767,9 +770,48 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -792,45 +834,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1152,56 +1155,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28" t="s">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="28"/>
+      <c r="H1" s="30"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="35" t="s">
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="30"/>
-      <c r="H3" s="36"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="49"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="34"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47"/>
       <c r="F4" s="12" t="s">
         <v>3</v>
       </c>
@@ -1213,22 +1216,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="47" t="s">
+      <c r="A5" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="48"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
-      <c r="F5" s="48"/>
-      <c r="G5" s="48"/>
-      <c r="H5" s="49"/>
+      <c r="B5" s="40"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="41"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="45" t="s">
+      <c r="B6" s="37" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1251,8 +1254,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="38"/>
-      <c r="B7" s="46"/>
+      <c r="A7" s="29"/>
+      <c r="B7" s="38"/>
       <c r="C7" s="19" t="s">
         <v>13</v>
       </c>
@@ -1308,16 +1311,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="41"/>
+      <c r="B8" s="32"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="33"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1823,16 +1826,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="42" t="s">
+      <c r="A19" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="43"/>
-      <c r="C19" s="43"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="43"/>
-      <c r="F19" s="43"/>
-      <c r="G19" s="43"/>
-      <c r="H19" s="44"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="35"/>
+      <c r="G19" s="35"/>
+      <c r="H19" s="36"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1964,8 +1967,8 @@
       <c r="AQ21"/>
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="9"/>
-      <c r="B22" s="8"/>
+      <c r="A22" s="14"/>
+      <c r="B22" s="14"/>
       <c r="C22" s="14"/>
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
@@ -2189,16 +2192,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="42" t="s">
+      <c r="A27" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="43"/>
-      <c r="C27" s="43"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="44"/>
+      <c r="B27" s="35"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35"/>
+      <c r="H27" s="36"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2424,10 +2427,13 @@
       <c r="AQ31"/>
     </row>
     <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="9" t="s">
+        <v>41</v>
+      </c>
       <c r="B32" s="8"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
       <c r="F32" s="14"/>
       <c r="G32" s="14"/>
       <c r="H32" s="15"/>
@@ -2650,6 +2656,11 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2657,11 +2668,6 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2672,12 +2678,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="02ab52c2-13d4-475f-b11b-1abd8b9844fa" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9336579e-41a2-4e28-b381-0917067c5e4b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2888,20 +2896,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="02ab52c2-13d4-475f-b11b-1abd8b9844fa" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9336579e-41a2-4e28-b381-0917067c5e4b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAD7F43D-D545-4C62-B92C-5979BC5339EF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E104E0C-D545-4F6B-9B75-6F88F0795FDB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="02ab52c2-13d4-475f-b11b-1abd8b9844fa"/>
+    <ds:schemaRef ds:uri="9336579e-41a2-4e28-b381-0917067c5e4b"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2926,12 +2935,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E104E0C-D545-4F6B-9B75-6F88F0795FDB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAD7F43D-D545-4C62-B92C-5979BC5339EF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="02ab52c2-13d4-475f-b11b-1abd8b9844fa"/>
-    <ds:schemaRef ds:uri="9336579e-41a2-4e28-b381-0917067c5e4b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>